<commit_message>
Update quick_demo fitting sheet: use RC0183/RC0197 to match Dollop groups
The chip's Dollop print map uses RC0183 (capture) and RC0197 (negative
control), not RC0358/RC0343. Updated fitting_protocol_sheet.xlsx and
uploaded to S3.

Made-with: Cursor
</commit_message>
<xml_diff>
--- a/config/calibration_data/quick_demo/v1.0/fitting_protocol_sheet.xlsx
+++ b/config/calibration_data/quick_demo/v1.0/fitting_protocol_sheet.xlsx
@@ -559,12 +559,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>RC0358</t>
+          <t>RC0183</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>RC0343</t>
+          <t>RC0197</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -648,7 +648,6 @@
           <t>None</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>